<commit_message>
UI Test Updated to multiple products
</commit_message>
<xml_diff>
--- a/test-data/ui-test-data/testData.xlsx
+++ b/test-data/ui-test-data/testData.xlsx
@@ -5,17 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WorkSpace\ecommerce_shopfy\test-data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WorkSpace\ecommerce_shopfy\test-data\ui-test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD160EE6-1C6C-419C-ACA0-0B1817D81A15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66E4FFCC-20B2-4618-985C-7D9DF9A4FA75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="register" sheetId="1" r:id="rId1"/>
     <sheet name="login" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
+    <sheet name="review" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="53">
   <si>
     <t>Name</t>
   </si>
@@ -146,7 +146,46 @@
     <t>gvvtest1</t>
   </si>
   <si>
-    <t>Quantity</t>
+    <t>Comments</t>
+  </si>
+  <si>
+    <t>ProductName</t>
+  </si>
+  <si>
+    <t>Blue Top</t>
+  </si>
+  <si>
+    <t>Men Tshirt</t>
+  </si>
+  <si>
+    <t>Printed Off Shoulder Top - White</t>
+  </si>
+  <si>
+    <t>Prasad</t>
+  </si>
+  <si>
+    <t>Jack</t>
+  </si>
+  <si>
+    <t>Roy</t>
+  </si>
+  <si>
+    <t>prasad@gmail.com</t>
+  </si>
+  <si>
+    <t>jack@gmail.com</t>
+  </si>
+  <si>
+    <t>roy@gmail.com</t>
+  </si>
+  <si>
+    <t>Good</t>
+  </si>
+  <si>
+    <t>Bad</t>
+  </si>
+  <si>
+    <t>Nice</t>
   </si>
 </sst>
 </file>
@@ -725,10 +764,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE99E6B8-824C-4732-B2C5-23DC1F2D6217}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="27.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.77734375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -736,13 +780,84 @@
         <v>2</v>
       </c>
       <c r="C1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1" t="s">
         <v>0</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" t="s">
         <v>39</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F4" t="s">
+        <v>52</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{E1BB2C22-6FBB-4EA9-8B24-76F5BD39B51C}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{4A5FB6CE-602C-4F01-ADB9-435BBA1980B3}"/>
+    <hyperlink ref="E4" r:id="rId3" xr:uid="{48BA9340-BD9D-442E-B625-22A3A4E5562D}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
TC updated to multiple & bat file added for jenkins
</commit_message>
<xml_diff>
--- a/test-data/ui-test-data/testData.xlsx
+++ b/test-data/ui-test-data/testData.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WorkSpace\ecommerce_shopfy\test-data\ui-test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66E4FFCC-20B2-4618-985C-7D9DF9A4FA75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDA16D7D-AB68-4937-B805-EB78E38F32D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="register" sheetId="1" r:id="rId1"/>
     <sheet name="login" sheetId="2" r:id="rId2"/>
     <sheet name="review" sheetId="3" r:id="rId3"/>
+    <sheet name="products" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="54">
   <si>
     <t>Name</t>
   </si>
@@ -186,6 +187,9 @@
   </si>
   <si>
     <t>Nice</t>
+  </si>
+  <si>
+    <t>Quantity</t>
   </si>
 </sst>
 </file>
@@ -663,6 +667,9 @@
       <c r="E3" t="s">
         <v>5</v>
       </c>
+      <c r="F3" t="s">
+        <v>24</v>
+      </c>
       <c r="G3">
         <v>23</v>
       </c>
@@ -860,4 +867,70 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EFE6B1D-A80A-40DB-85CF-EA6EBD9037B2}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>